<commit_message>
Add project presentation and requirements file; update output files
- Created a new presentation document detailing the FIFA WC Predictor project, including purpose, structure, dependencies, and workflow.
- Added a requirements.txt file listing necessary libraries for the project.
- Updated several output files including images and Excel sheets to reflect the latest analysis and predictions.
</commit_message>
<xml_diff>
--- a/output_powerbi/top4_modelo_ml.xlsx
+++ b/output_powerbi/top4_modelo_ml.xlsx
@@ -470,16 +470,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>40.3</v>
+        <v>31.8</v>
       </c>
       <c r="C2" t="n">
-        <v>17.6</v>
+        <v>13.8</v>
       </c>
       <c r="D2" t="n">
-        <v>18</v>
+        <v>13.3</v>
       </c>
       <c r="E2" t="n">
-        <v>7.4</v>
+        <v>5.7</v>
       </c>
       <c r="F2" t="n">
         <v>15</v>
@@ -497,20 +497,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Espana</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>34.4</v>
+        <v>20.2</v>
       </c>
       <c r="C3" t="n">
-        <v>37.7</v>
+        <v>31.5</v>
       </c>
       <c r="D3" t="n">
-        <v>17.3</v>
+        <v>21.1</v>
       </c>
       <c r="E3" t="n">
-        <v>10.7</v>
+        <v>27.2</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -528,20 +528,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Espana</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13.3</v>
+        <v>19.7</v>
       </c>
       <c r="C4" t="n">
-        <v>14.6</v>
+        <v>28.6</v>
       </c>
       <c r="D4" t="n">
-        <v>43.7</v>
+        <v>23.8</v>
       </c>
       <c r="E4" t="n">
-        <v>28.4</v>
+        <v>27.9</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -559,20 +559,20 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Noruega</t>
+          <t>Inglaterra</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7.5</v>
+        <v>10.1</v>
       </c>
       <c r="C5" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="D5" t="n">
-        <v>12.3</v>
+        <v>17.2</v>
       </c>
       <c r="E5" t="n">
-        <v>32.5</v>
+        <v>16.3</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -590,20 +590,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Inglaterra</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3.1</v>
+        <v>9.4</v>
       </c>
       <c r="C6" t="n">
-        <v>7.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D6" t="n">
-        <v>5.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>12.2</v>
+        <v>8.4</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -621,20 +621,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Suiza</t>
+          <t>Noruega</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="C7" t="n">
-        <v>3.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>3.2</v>
+        <v>15.9</v>
       </c>
       <c r="E7" t="n">
-        <v>8.800000000000001</v>
+        <v>14.5</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>

</xml_diff>